<commit_message>
Physics 105 cap correction
</commit_message>
<xml_diff>
--- a/merged_course_schedule.xlsx
+++ b/merged_course_schedule.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\4. Horowitz Service\2. Advising\catalog-code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vhorowit\Documents\GitHub\Colleague_self_service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F427126-8D35-4DA7-8710-F9988D32E3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4654AE97-5DD5-4163-B9E2-D48A8ED74275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14754" uniqueCount="4118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14750" uniqueCount="4118">
   <si>
     <t>Subject Code</t>
   </si>
@@ -60055,18 +60055,6 @@
       <c r="AY519">
         <v>40</v>
       </c>
-      <c r="AZ519" t="s">
-        <v>129</v>
-      </c>
-      <c r="BA519" t="s">
-        <v>129</v>
-      </c>
-      <c r="BB519">
-        <v>10</v>
-      </c>
-      <c r="BC519">
-        <v>10</v>
-      </c>
       <c r="BD519" t="s">
         <v>81</v>
       </c>
@@ -60161,18 +60149,6 @@
       </c>
       <c r="AY520">
         <v>40</v>
-      </c>
-      <c r="AZ520" t="s">
-        <v>129</v>
-      </c>
-      <c r="BA520" t="s">
-        <v>129</v>
-      </c>
-      <c r="BB520">
-        <v>10</v>
-      </c>
-      <c r="BC520">
-        <v>10</v>
       </c>
       <c r="BD520" t="s">
         <v>81</v>

</xml_diff>

<commit_message>
Manually fixed some senior courses
</commit_message>
<xml_diff>
--- a/merged_course_schedule.xlsx
+++ b/merged_course_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vhorowit\Documents\GitHub\Colleague_self_service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4654AE97-5DD5-4163-B9E2-D48A8ED74275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{414AA0D7-8630-489E-B6F9-04AFA0123DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61892,13 +61892,13 @@
         <v>1</v>
       </c>
       <c r="BD543" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE543" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF543" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG543" t="s">
         <v>81</v>
@@ -61981,13 +61981,13 @@
         <v>1</v>
       </c>
       <c r="BD544" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE544" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF544" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG544" t="s">
         <v>81</v>
@@ -62251,13 +62251,13 @@
         <v>1</v>
       </c>
       <c r="BD547" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE547" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF547" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG547" t="s">
         <v>81</v>
@@ -69434,14 +69434,16 @@
       <c r="BG623" t="s">
         <v>81</v>
       </c>
-      <c r="BH623" t="s">
+      <c r="BH623" s="2" t="s">
         <v>4117</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="BH15" r:id="rId1" location="middle" xr:uid="{8EEF2D64-E1EE-4C4D-BE15-343966B2291C}"/>
+    <hyperlink ref="BH623" r:id="rId2" xr:uid="{2CBC0E25-1319-4A5F-B01A-4C19F9784136}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added some of the missing weblinks to smartcatalogue
</commit_message>
<xml_diff>
--- a/merged_course_schedule.xlsx
+++ b/merged_course_schedule.xlsx
@@ -8,15 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vhorowit\Documents\GitHub\Colleague_self_service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{414AA0D7-8630-489E-B6F9-04AFA0123DE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512D4FB7-A8EA-4438-A103-E0123916271D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16320" yWindow="-12690" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14750" uniqueCount="4118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14765" uniqueCount="4122">
   <si>
     <t>Subject Code</t>
   </si>
@@ -12379,13 +12388,25 @@
   </si>
   <si>
     <t>https://hamilton.smartcatalogiq.com/en/current/college-catalogue/courses/wmgst-womens-and-gender-studies/400/wmgst-405</t>
+  </si>
+  <si>
+    <t>https://hamilton.smartcatalogiq.com/en/current/college-catalogue/courses/afrst-africana-studies/200-300/afrst-267367</t>
+  </si>
+  <si>
+    <t>https://hamilton.smartcatalogiq.com/en/current/college-catalogue/courses/geosc-geosciences/510500/geosc-510-511</t>
+  </si>
+  <si>
+    <t>https://hamilton.smartcatalogiq.com/en/current/college-catalogue/courses/ltam-latin-american-and-latine-studies/100-200/ltam-165</t>
+  </si>
+  <si>
+    <t>https://hamilton.smartcatalogiq.com/en/current/college-catalogue/courses/thetr-theatre/100/thetr-141-142</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -12397,14 +12418,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -12439,19 +12452,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -12933,7 +12943,7 @@
       <c r="BG1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BH1" t="s">
         <v>59</v>
       </c>
     </row>
@@ -13616,6 +13626,9 @@
       <c r="BG8" t="s">
         <v>81</v>
       </c>
+      <c r="BH8" t="s">
+        <v>4118</v>
+      </c>
     </row>
     <row r="9" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -13803,6 +13816,9 @@
       <c r="BG10" t="s">
         <v>81</v>
       </c>
+      <c r="BH10" t="s">
+        <v>4118</v>
+      </c>
     </row>
     <row r="11" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -14263,7 +14279,7 @@
       <c r="BG15" t="s">
         <v>81</v>
       </c>
-      <c r="BH15" s="2" t="s">
+      <c r="BH15" t="s">
         <v>221</v>
       </c>
     </row>
@@ -14462,6 +14478,9 @@
       <c r="BG17" t="s">
         <v>81</v>
       </c>
+      <c r="BH17" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="18" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -14872,6 +14891,9 @@
       <c r="BG21" t="s">
         <v>81</v>
       </c>
+      <c r="BH21" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="22" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -38251,6 +38273,9 @@
       <c r="BG282" t="s">
         <v>81</v>
       </c>
+      <c r="BH282" t="s">
+        <v>4119</v>
+      </c>
     </row>
     <row r="283" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A283" t="s">
@@ -38331,6 +38356,9 @@
       <c r="BG283" t="s">
         <v>81</v>
       </c>
+      <c r="BH283" t="s">
+        <v>4119</v>
+      </c>
     </row>
     <row r="284" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A284" t="s">
@@ -38411,6 +38439,9 @@
       <c r="BG284" t="s">
         <v>81</v>
       </c>
+      <c r="BH284" t="s">
+        <v>4119</v>
+      </c>
     </row>
     <row r="285" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A285" t="s">
@@ -38491,6 +38522,9 @@
       <c r="BG285" t="s">
         <v>81</v>
       </c>
+      <c r="BH285" t="s">
+        <v>4119</v>
+      </c>
     </row>
     <row r="286" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A286" t="s">
@@ -38571,6 +38605,9 @@
       <c r="BG286" t="s">
         <v>81</v>
       </c>
+      <c r="BH286" t="s">
+        <v>4119</v>
+      </c>
     </row>
     <row r="287" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A287" t="s">
@@ -47060,6 +47097,9 @@
       <c r="BG377" t="s">
         <v>81</v>
       </c>
+      <c r="BH377" t="s">
+        <v>2654</v>
+      </c>
     </row>
     <row r="378" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A378" t="s">
@@ -47143,6 +47183,9 @@
       <c r="BG378" t="s">
         <v>81</v>
       </c>
+      <c r="BH378" t="s">
+        <v>2660</v>
+      </c>
     </row>
     <row r="379" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A379" t="s">
@@ -47229,6 +47272,9 @@
       <c r="BG379" t="s">
         <v>81</v>
       </c>
+      <c r="BH379" t="s">
+        <v>2667</v>
+      </c>
     </row>
     <row r="380" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A380" t="s">
@@ -51250,6 +51296,9 @@
       <c r="BG423" t="s">
         <v>81</v>
       </c>
+      <c r="BH423" t="s">
+        <v>4120</v>
+      </c>
     </row>
     <row r="424" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A424" t="s">
@@ -51437,6 +51486,9 @@
       <c r="BG425" t="s">
         <v>81</v>
       </c>
+      <c r="BH425" t="s">
+        <v>4120</v>
+      </c>
     </row>
     <row r="426" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A426" t="s">
@@ -67706,6 +67758,9 @@
       <c r="BG605" t="s">
         <v>81</v>
       </c>
+      <c r="BH605" t="s">
+        <v>4121</v>
+      </c>
     </row>
     <row r="606" spans="1:60" x14ac:dyDescent="0.35">
       <c r="A606" t="s">
@@ -69434,16 +69489,12 @@
       <c r="BG623" t="s">
         <v>81</v>
       </c>
-      <c r="BH623" s="2" t="s">
+      <c r="BH623" t="s">
         <v>4117</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="BH15" r:id="rId1" location="middle" xr:uid="{8EEF2D64-E1EE-4C4D-BE15-343966B2291C}"/>
-    <hyperlink ref="BH623" r:id="rId2" xr:uid="{2CBC0E25-1319-4A5F-B01A-4C19F9784136}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Manually set all senior courses to be for seniors
</commit_message>
<xml_diff>
--- a/merged_course_schedule.xlsx
+++ b/merged_course_schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vhorowit\Documents\GitHub\Colleague_self_service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512D4FB7-A8EA-4438-A103-E0123916271D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306C296E-2407-470B-92AA-A137DC0B1723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-12690" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -12418,6 +12418,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -16666,13 +16667,13 @@
         <v>1</v>
       </c>
       <c r="BD41" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE41" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF41" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG41" t="s">
         <v>81</v>
@@ -20917,13 +20918,13 @@
         <v>1</v>
       </c>
       <c r="BD86" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE86" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF86" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG86" t="s">
         <v>81</v>
@@ -21006,13 +21007,13 @@
         <v>1</v>
       </c>
       <c r="BD87" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE87" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF87" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG87" t="s">
         <v>81</v>
@@ -21095,13 +21096,13 @@
         <v>1</v>
       </c>
       <c r="BD88" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE88" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF88" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG88" t="s">
         <v>81</v>
@@ -21184,13 +21185,13 @@
         <v>1</v>
       </c>
       <c r="BD89" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE89" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF89" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG89" t="s">
         <v>81</v>
@@ -21273,13 +21274,13 @@
         <v>1</v>
       </c>
       <c r="BD90" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE90" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF90" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG90" t="s">
         <v>81</v>
@@ -21362,13 +21363,13 @@
         <v>1</v>
       </c>
       <c r="BD91" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE91" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF91" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG91" t="s">
         <v>81</v>
@@ -24358,13 +24359,13 @@
         <v>1</v>
       </c>
       <c r="BD128" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE128" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF128" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG128" t="s">
         <v>81</v>
@@ -24438,13 +24439,13 @@
         <v>1</v>
       </c>
       <c r="BD129" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE129" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF129" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG129" t="s">
         <v>81</v>
@@ -24518,13 +24519,13 @@
         <v>1</v>
       </c>
       <c r="BD130" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE130" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF130" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG130" t="s">
         <v>81</v>
@@ -34920,13 +34921,13 @@
         <v>1</v>
       </c>
       <c r="BD246" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE246" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF246" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG246" t="s">
         <v>81</v>
@@ -38262,13 +38263,13 @@
         <v>1</v>
       </c>
       <c r="BD282" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE282" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF282" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG282" t="s">
         <v>81</v>
@@ -38345,13 +38346,13 @@
         <v>1</v>
       </c>
       <c r="BD283" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE283" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF283" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG283" t="s">
         <v>81</v>
@@ -38428,13 +38429,13 @@
         <v>1</v>
       </c>
       <c r="BD284" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE284" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF284" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG284" t="s">
         <v>81</v>
@@ -38511,13 +38512,13 @@
         <v>1</v>
       </c>
       <c r="BD285" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE285" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF285" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG285" t="s">
         <v>81</v>
@@ -38594,13 +38595,13 @@
         <v>1</v>
       </c>
       <c r="BD286" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE286" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF286" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG286" t="s">
         <v>81</v>
@@ -39110,13 +39111,13 @@
         <v>1</v>
       </c>
       <c r="BD292" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE292" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF292" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG292" t="s">
         <v>81</v>

</xml_diff>

<commit_message>
1 more senior course, manually categorized
</commit_message>
<xml_diff>
--- a/merged_course_schedule.xlsx
+++ b/merged_course_schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vhorowit\Documents\GitHub\Colleague_self_service\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306C296E-2407-470B-92AA-A137DC0B1723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1CC1E7-E63E-45DE-A0C5-5D976B870EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1810" yWindow="2470" windowWidth="14400" windowHeight="8180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -15783,13 +15783,13 @@
         <v>1</v>
       </c>
       <c r="BD31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BE31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BF31" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="BG31" t="s">
         <v>81</v>

</xml_diff>